<commit_message>
refactor: improve freight tracking, group external loads, update driver excel sheet and gitignore
</commit_message>
<xml_diff>
--- a/public/Dados Motoristas.xlsx
+++ b/public/Dados Motoristas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DEV\MIDAS RENT A CAR\midas-log\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00AC6AE5-836B-41D6-86A1-AC529CECCE39}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D662904-5CF0-4A8F-962D-CF293255B0F8}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{787D443B-6186-4946-A670-5DA3C1446C88}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="231">
   <si>
     <t xml:space="preserve"> CPF</t>
   </si>
@@ -707,6 +707,24 @@
   </si>
   <si>
     <t>NQL6A96</t>
+  </si>
+  <si>
+    <t>ANASTACIO TIBURCIO DA COSTA JUNIOR</t>
+  </si>
+  <si>
+    <t>OSI1413</t>
+  </si>
+  <si>
+    <t>GERMANO CAVALCANTE CEZAR</t>
+  </si>
+  <si>
+    <t>KDZ3550</t>
+  </si>
+  <si>
+    <t>JOAO LENON SILVA SALES</t>
+  </si>
+  <si>
+    <t>055082733</t>
   </si>
 </sst>
 </file>
@@ -1352,8 +1370,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CDBBDD53-C0F0-4D69-BB2A-7A12F8DAE60F}" name="Tabela1" displayName="Tabela1" ref="A1:I62" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10" tableBorderDxfId="9">
-  <autoFilter ref="A1:I62" xr:uid="{CDBBDD53-C0F0-4D69-BB2A-7A12F8DAE60F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CDBBDD53-C0F0-4D69-BB2A-7A12F8DAE60F}" name="Tabela1" displayName="Tabela1" ref="A1:I65" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10" tableBorderDxfId="9">
+  <autoFilter ref="A1:I65" xr:uid="{CDBBDD53-C0F0-4D69-BB2A-7A12F8DAE60F}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{520F8D1D-FD72-4AFB-9FC5-7D74F8E1C644}" name="NATUREZA" dataDxfId="8"/>
     <tableColumn id="2" xr3:uid="{1637597A-386A-4B10-ACA3-751188B9BC58}" name="PLACA" dataDxfId="7"/>
@@ -1666,7 +1684,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73C36CC1-71FE-44C6-8B99-4ADD2229EA60}">
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:I65"/>
   <sheetFormatPr defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -3452,26 +3470,95 @@
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A62" s="11" t="s">
-        <v>178</v>
+        <v>50</v>
       </c>
       <c r="B62" s="11" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="C62" s="11" t="s">
         <v>19</v>
       </c>
       <c r="D62" s="12">
-        <v>13400</v>
+        <v>13260</v>
       </c>
       <c r="E62" s="11" t="s">
-        <v>223</v>
-      </c>
-      <c r="F62" s="21">
-        <v>31076416349</v>
-      </c>
+        <v>225</v>
+      </c>
+      <c r="F62" s="21"/>
       <c r="G62" s="11"/>
       <c r="H62" s="11"/>
       <c r="I62" s="14"/>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A63" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="B63" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="C63" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="D63" s="12">
+        <v>19000</v>
+      </c>
+      <c r="E63" s="11" t="s">
+        <v>227</v>
+      </c>
+      <c r="F63" s="21">
+        <v>68894724387</v>
+      </c>
+      <c r="G63" s="11"/>
+      <c r="H63" s="11"/>
+      <c r="I63" s="14" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A64" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="B64" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="C64" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="D64" s="12"/>
+      <c r="E64" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="F64" s="21">
+        <v>74628623104</v>
+      </c>
+      <c r="G64" s="11"/>
+      <c r="H64" s="11"/>
+      <c r="I64" s="14" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A65" s="11" t="s">
+        <v>178</v>
+      </c>
+      <c r="B65" s="11" t="s">
+        <v>222</v>
+      </c>
+      <c r="C65" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="D65" s="12">
+        <v>13400</v>
+      </c>
+      <c r="E65" s="11" t="s">
+        <v>223</v>
+      </c>
+      <c r="F65" s="21">
+        <v>31076416349</v>
+      </c>
+      <c r="G65" s="11"/>
+      <c r="H65" s="11"/>
+      <c r="I65" s="14"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:H13">

</xml_diff>

<commit_message>
feat: implement closed months functionality and lock freight romaneios edits
</commit_message>
<xml_diff>
--- a/public/Dados Motoristas.xlsx
+++ b/public/Dados Motoristas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DEV\MIDAS RENT A CAR\midas-log\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0B14F20-6282-4AD3-A170-9EDFF474F1FD}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{705358E7-0AC8-4193-ADFB-CCFA7626B916}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{787D443B-6186-4946-A670-5DA3C1446C88}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="251">
   <si>
     <t xml:space="preserve"> CPF</t>
   </si>
@@ -779,6 +779,12 @@
   </si>
   <si>
     <t>FRANCISCO ANTONIO DE SOUSA SILVA</t>
+  </si>
+  <si>
+    <t>POE5E12</t>
+  </si>
+  <si>
+    <t>WANDERSON GONCALVES DA SILVA</t>
   </si>
 </sst>
 </file>
@@ -905,7 +911,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1002,6 +1008,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1445,8 +1454,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CDBBDD53-C0F0-4D69-BB2A-7A12F8DAE60F}" name="Tabela1" displayName="Tabela1" ref="A1:I72" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10" tableBorderDxfId="9">
-  <autoFilter ref="A1:I72" xr:uid="{CDBBDD53-C0F0-4D69-BB2A-7A12F8DAE60F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CDBBDD53-C0F0-4D69-BB2A-7A12F8DAE60F}" name="Tabela1" displayName="Tabela1" ref="A1:I73" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10" tableBorderDxfId="9">
+  <autoFilter ref="A1:I73" xr:uid="{CDBBDD53-C0F0-4D69-BB2A-7A12F8DAE60F}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{520F8D1D-FD72-4AFB-9FC5-7D74F8E1C644}" name="NATUREZA" dataDxfId="8"/>
     <tableColumn id="2" xr3:uid="{1637597A-386A-4B10-ACA3-751188B9BC58}" name="PLACA" dataDxfId="7"/>
@@ -1759,7 +1768,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73C36CC1-71FE-44C6-8B99-4ADD2229EA60}">
-  <dimension ref="A1:I72"/>
+  <dimension ref="A1:I73"/>
   <sheetFormatPr defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -3811,6 +3820,29 @@
       <c r="I72" s="14" t="s">
         <v>149</v>
       </c>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A73" s="31" t="s">
+        <v>50</v>
+      </c>
+      <c r="B73" s="31" t="s">
+        <v>249</v>
+      </c>
+      <c r="C73" s="31" t="s">
+        <v>21</v>
+      </c>
+      <c r="D73" s="32">
+        <v>30473</v>
+      </c>
+      <c r="E73" s="31" t="s">
+        <v>250</v>
+      </c>
+      <c r="F73" s="33">
+        <v>950626376</v>
+      </c>
+      <c r="G73" s="31"/>
+      <c r="H73" s="31"/>
+      <c r="I73" s="34"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:H13">

</xml_diff>